<commit_message>
Add favicon, Open Graph tags, and WhatsApp share button to all pages
</commit_message>
<xml_diff>
--- a/לוח זמנים אמא.xlsx
+++ b/לוח זמנים אמא.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davidhai\יום הולדת אמא\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2249F86E-44BC-47B8-A8E6-8E5AEFEB7154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57C76B4-530E-4F8B-B339-744C6230AAC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8E9FB3A8-0EEF-4272-A0E1-FF7076610F86}"/>
+    <workbookView xWindow="1125" yWindow="4305" windowWidth="21600" windowHeight="11175" xr2:uid="{8E9FB3A8-0EEF-4272-A0E1-FF7076610F86}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
   <si>
     <t>לידה</t>
   </si>
@@ -677,6 +677,9 @@
       <c r="B6" t="s">
         <v>39</v>
       </c>
+      <c r="E6" t="s">
+        <v>58</v>
+      </c>
       <c r="F6" t="s">
         <v>44</v>
       </c>

</xml_diff>

<commit_message>
Music: cycle through multiple birthday tunes instead of only Happy Birthday
</commit_message>
<xml_diff>
--- a/לוח זמנים אמא.xlsx
+++ b/לוח זמנים אמא.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davidhai\יום הולדת אמא\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57C76B4-530E-4F8B-B339-744C6230AAC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60BFD3C1-E321-4899-AD9F-F6437392B738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1125" yWindow="4305" windowWidth="21600" windowHeight="11175" xr2:uid="{8E9FB3A8-0EEF-4272-A0E1-FF7076610F86}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="60">
   <si>
     <t>לידה</t>
   </si>
@@ -216,6 +216,9 @@
   </si>
   <si>
     <t>V</t>
+  </si>
+  <si>
+    <t>💛 יום הולדת 40 למוריה 💛</t>
   </si>
 </sst>
 </file>
@@ -629,6 +632,9 @@
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="H3" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -854,6 +860,7 @@
     <hyperlink ref="H8" r:id="rId4" display="https://davidhaiintel.github.io/David-Hai-Cohen/couple.html" xr:uid="{CCAF763B-C9AD-4D52-A072-38918D161DDC}"/>
     <hyperlink ref="H7" r:id="rId5" display="https://davidhaiintel.github.io/David-Hai-Cohen/parenting.html" xr:uid="{E8B435B9-3B0D-4F5E-A2F5-35AE22C9ABF1}"/>
     <hyperlink ref="H4" r:id="rId6" display="https://davidhaiintel.github.io/David-Hai-Cohen/recipes.html" xr:uid="{9B7037BB-0126-45E3-B676-C43B41BE13FB}"/>
+    <hyperlink ref="H3" r:id="rId7" display="https://davidhaiintel.github.io/David-Hai-Cohen/index.html" xr:uid="{120ADC74-94D3-497D-A6E1-D348D2651DF9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>